<commit_message>
Normalize conference names and clean player pool
</commit_message>
<xml_diff>
--- a/ALL_NBA_PLAYERS.xlsx
+++ b/ALL_NBA_PLAYERS.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C473"/>
+  <dimension ref="A1:C471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,7 +475,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MVC</t>
+          <t>Missouri Valley Conference</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MVC</t>
+          <t>Missouri Valley Conference</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>MVC</t>
+          <t>Missouri Valley Conference</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>AAC</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>The American</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>AAC</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>AAC</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
@@ -3144,7 +3144,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Mountain East Conference</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>MVC</t>
+          <t>Missouri Valley Conference</t>
         </is>
       </c>
     </row>
@@ -3586,7 +3586,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>AAC</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -3688,7 +3688,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3773,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
@@ -4392,522 +4392,522 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Jonas Valančiūnas</t>
+          <t>Jonathan Isaac</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Lietuvos rytas Vilnius</t>
+          <t>Florida State</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Jonathan Isaac</t>
+          <t>Jonathan Mogbo</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Florida State</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Jonathan Mogbo</t>
+          <t>Jordan Clarkson</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Missouri</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Jordan Clarkson</t>
+          <t>Jordan Goodwin</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>St. Louis</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Atlantic 10</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Jordan Goodwin</t>
+          <t>Jordan Hawkins</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>St. Louis</t>
+          <t>Connecticut</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Atlantic 10</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Jordan Hawkins</t>
+          <t>Jordan McLaughlin</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Connecticut</t>
+          <t>USC</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Jordan McLaughlin</t>
+          <t>Jordan Miller</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>USC</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Jordan Miller</t>
+          <t>Jordan Poole</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Michigan</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Jordan Poole</t>
+          <t>Jordan Walsh</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Jordan Walsh</t>
+          <t>Jose Alvarado</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Georgia Tech</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Jose Alvarado</t>
+          <t>Josh Green</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Georgia Tech</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Josh Green</t>
+          <t>Josh Hart</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Villanova</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Josh Hart</t>
+          <t>Josh Minott</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Villanova</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Josh Minott</t>
+          <t>Josh Oduro</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Providence</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>AAC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Josh Oduro</t>
+          <t>Josh Okogie</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Providence</t>
+          <t>Georgia Tech</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Josh Okogie</t>
+          <t>Jrue Holiday</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Georgia Tech</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Jrue Holiday</t>
+          <t>Julian Champagnie</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>St. John's</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Julian Champagnie</t>
+          <t>Julian Phillips</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>St. John's</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Julian Phillips</t>
+          <t>Julian Reese</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>Maryland</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Julian Reese</t>
+          <t>Julian Strawther</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Maryland</t>
+          <t>Gonzaga</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Julian Strawther</t>
+          <t>Julius Randle</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Gonzaga</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Julius Randle</t>
+          <t>Justin Champagnie</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Justin Champagnie</t>
+          <t>Justin Edwards</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Justin Edwards</t>
+          <t>KJ Simpson</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Colorado</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>KJ Simpson</t>
+          <t>Kam Jones</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Colorado</t>
+          <t>Marquette</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Kam Jones</t>
+          <t>Karl-Anthony Towns</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Marquette</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Karl-Anthony Towns</t>
+          <t>Kasparas Jakučionis</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Illinois</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Kasparas Jakučionis</t>
+          <t>Kawhi Leonard</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Illinois</t>
+          <t>San Diego State</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Mountain West</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Kawhi Leonard</t>
+          <t>Keaton Wallace</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>San Diego State</t>
+          <t>UTSA</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Mountain West</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Keaton Wallace</t>
+          <t>Keegan Murray</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>UTSA</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>American Athletic Conference</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Keegan Murray</t>
+          <t>Kel'el Ware</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>Indiana</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -4919,114 +4919,114 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Kel'el Ware</t>
+          <t>Keldon Johnson</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Keldon Johnson</t>
+          <t>Kelly Olynyk</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Gonzaga</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Kelly Olynyk</t>
+          <t>Kelly Oubre Jr.</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Gonzaga</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Kelly Oubre Jr.</t>
+          <t>Kennedy Chandler</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Kennedy Chandler</t>
+          <t>Kenrich Williams</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>TCU</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Kenrich Williams</t>
+          <t>Kentavious Caldwell-Pope</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>TCU</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Kentavious Caldwell-Pope</t>
+          <t>Keon Ellis</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Alabama</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -5038,29 +5038,29 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Keon Ellis</t>
+          <t>Keshad Johnson</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Keshad Johnson</t>
+          <t>Keshon Gilbert</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Iowa State</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -5072,46 +5072,46 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Keshon Gilbert</t>
+          <t>Kevin Durant</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Iowa State</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Kevin Durant</t>
+          <t>Kevin Huerter</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Maryland</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Kevin Huerter</t>
+          <t>Kevin Love</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Maryland</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -5123,46 +5123,46 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Kevin Love</t>
+          <t>Kevin McCullar Jr.</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Kevin McCullar Jr.</t>
+          <t>Kevin Porter Jr.</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>USC</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Kevin Porter Jr.</t>
+          <t>Kevon Looney</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>USC</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -5174,199 +5174,199 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Kevon Looney</t>
+          <t>Keyonte George</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Baylor</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Keyonte George</t>
+          <t>Khaman Maluach</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Baylor</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Khaman Maluach</t>
+          <t>Khris Middleton</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Texas A&amp;M</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Khris Middleton</t>
+          <t>Klay Thompson</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Texas A&amp;M</t>
+          <t>Washington State</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Pac-12</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Klay Thompson</t>
+          <t>Kobe Brown</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Washington State</t>
+          <t>Missouri</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Pac-12</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Kobe Brown</t>
+          <t>Kobe Bufkin</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>Michigan</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Kobe Bufkin</t>
+          <t>Kobe Sanders</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Nevada</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Mountain West</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Kobe Sanders</t>
+          <t>Koby Brea</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Nevada</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Mountain West</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Koby Brea</t>
+          <t>Kon Knueppel</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Kon Knueppel</t>
+          <t>Kris Dunn</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Providence</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Kris Dunn</t>
+          <t>Kris Murray</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Providence</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Kris Murray</t>
+          <t>Kyle Anderson</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -5378,80 +5378,80 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Kyle Anderson</t>
+          <t>Kyle Filipowski</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Kyle Filipowski</t>
+          <t>Kyle Kuzma</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Utah</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Kyle Kuzma</t>
+          <t>Kyle Lowry</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Villanova</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Kyle Lowry</t>
+          <t>Kyrie Irving</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Villanova</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Kyrie Irving</t>
+          <t>Kyshawn George</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -5463,301 +5463,301 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Kyshawn George</t>
+          <t>LJ Cryer</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>LJ Cryer</t>
+          <t>Landry Shamet</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Wichita State</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Landry Shamet</t>
+          <t>Larry Nance Jr.</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Wichita State</t>
+          <t>Wyoming</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>AAC</t>
+          <t>Mountain West</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Larry Nance Jr.</t>
+          <t>Lauri Markkanen</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Wyoming</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Mountain West</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Lauri Markkanen</t>
+          <t>Leaky Black</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Leaky Black</t>
+          <t>Liam McNeeley</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>Connecticut</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Liam McNeeley</t>
+          <t>Lindy Waters III</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Connecticut</t>
+          <t>Oklahoma State</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Lindy Waters III</t>
+          <t>Lucas Williamson</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Oklahoma State</t>
+          <t>Loyola-Chicago</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Atlantic 10</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Lucas Williamson</t>
+          <t>Luguentz Dort</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Loyola-Chicago</t>
+          <t>Arizona State</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Atlantic 10</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Luguentz Dort</t>
+          <t>Luka Garza</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Arizona State</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Luka Garza</t>
+          <t>Luke Kennard</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Luke Kennard</t>
+          <t>Luke Kornet</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Luke Kornet</t>
+          <t>Mac McClung</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>Texas Tech</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Mac McClung</t>
+          <t>Malachi Smith</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Texas Tech</t>
+          <t>Gonzaga</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Malachi Smith</t>
+          <t>Malevy Leons</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Gonzaga</t>
+          <t>Bradley</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>Missouri Valley Conference</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Malevy Leons</t>
+          <t>Malik Monk</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Bradley</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>MVC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Malik Monk</t>
+          <t>Marcus Sasser</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Marcus Sasser</t>
+          <t>Marcus Smart</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Oklahoma State</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -5769,58 +5769,58 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Marcus Smart</t>
+          <t>Mark Williams</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Oklahoma State</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Mark Williams</t>
+          <t>Markelle Fultz</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Washington</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Markelle Fultz</t>
+          <t>Marvin Bagley III</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Marvin Bagley III</t>
+          <t>Mason Plumlee</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -5837,29 +5837,29 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Mason Plumlee</t>
+          <t>Matisse Thybulle</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Washington</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Matisse Thybulle</t>
+          <t>Max Christie</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Michigan State</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -5871,148 +5871,148 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Max Christie</t>
+          <t>Max Shulga</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Michigan State</t>
+          <t>VCU</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Atlantic 10</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Max Shulga</t>
+          <t>Max Strus</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>VCU</t>
+          <t>DePaul</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Atlantic 10</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Max Strus</t>
+          <t>Maxime Raynaud</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>DePaul</t>
+          <t>Stanford</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Maxime Raynaud</t>
+          <t>Micah Peavy</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Stanford</t>
+          <t>Georgetown</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Micah Peavy</t>
+          <t>Micah Potter</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Georgetown</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Micah Potter</t>
+          <t>Michael Porter Jr.</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>Missouri</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>Michael Porter Jr.</t>
+          <t>Mikal Bridges</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>Villanova</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>Mikal Bridges</t>
+          <t>Mike Conley</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Villanova</t>
+          <t>Ohio State</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>Mike Conley</t>
+          <t>Miles Bridges</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Ohio State</t>
+          <t>Michigan State</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -6024,267 +6024,267 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Miles Bridges</t>
+          <t>Miles McBride</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Michigan State</t>
+          <t>West Virginia</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Miles McBride</t>
+          <t>Mitchell Robinson</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>West Virginia</t>
+          <t>Western Kentucky</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Conference USA</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Mitchell Robinson</t>
+          <t>Moritz Wagner</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Western Kentucky</t>
+          <t>Michigan</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Conference USA</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>Moritz Wagner</t>
+          <t>Moses Moody</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>Moses Moody</t>
+          <t>Mouhamed Gueye</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Washington State</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Pac-12</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>Mouhamed Gueye</t>
+          <t>Moussa Cisse</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Washington State</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Pac-12</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>Moussa Cisse</t>
+          <t>Moussa Diabaté</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Michigan</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>AAC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>Moussa Diabaté</t>
+          <t>Myles Turner</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Myles Turner</t>
+          <t>Myron Gardner</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Arkansas-Little Rock</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Ohio Valley</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>Myron Gardner</t>
+          <t>Nae'Qwan Tomlin</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Arkansas-Little Rock</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Ohio Valley</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>Nae'Qwan Tomlin</t>
+          <t>Naji Marshall</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Xavier</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>AAC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>Naji Marshall</t>
+          <t>Nate Williams</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Xavier</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Mid-American</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>Nate Williams</t>
+          <t>Naz Reid</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>LSU</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Mid-American</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>Naz Reid</t>
+          <t>Neemias Queta</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>LSU</t>
+          <t>Utah State</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Pac-12</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Neemias Queta</t>
+          <t>Nic Claxton</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Utah State</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Pac-12</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Nic Claxton</t>
+          <t>Nick Richards</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -6296,12 +6296,12 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>Nick Richards</t>
+          <t>Nick Smith Jr.</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -6313,262 +6313,262 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>Nick Smith Jr.</t>
+          <t>Nickeil Alexander-Walker</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Virginia Tech</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>Nickeil Alexander-Walker</t>
+          <t>Nikola Vučević</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Virginia Tech</t>
+          <t>USC</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>Nicolas Batum</t>
+          <t>Nique Clifford</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Le Mans</t>
+          <t>Colorado State</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Mountain West</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>Nikola Vučević</t>
+          <t>Noah Clowney</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>USC</t>
+          <t>Alabama</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>Nique Clifford</t>
+          <t>Norchad Omier</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Colorado State</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Mountain West</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>Noah Clowney</t>
+          <t>Norman Powell</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>Norchad Omier</t>
+          <t>OG Anunoby</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Indiana</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>Norman Powell</t>
+          <t>Obi Toppin</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Dayton</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Atlantic 10</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>OG Anunoby</t>
+          <t>Ochai Agbaji</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>Obi Toppin</t>
+          <t>Olivier Sarr</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Dayton</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Atlantic 10</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>Ochai Agbaji</t>
+          <t>Olivier-Maxence Prosper</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Marquette</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>Olivier Sarr</t>
+          <t>Omer Yurtseven</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Georgetown</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>Olivier-Maxence Prosper</t>
+          <t>Onyeka Okongwu</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Marquette</t>
+          <t>USC</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>Omer Yurtseven</t>
+          <t>Oscar Tshiebwe</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Georgetown</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>Onyeka Okongwu</t>
+          <t>Oso Ighodaro</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>USC</t>
+          <t>Marquette</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>Oscar Tshiebwe</t>
+          <t>P.J. Washington</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -6585,63 +6585,63 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>Oso Ighodaro</t>
+          <t>PJ Hall</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Marquette</t>
+          <t>Clemson</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>P.J. Washington</t>
+          <t>Paolo Banchero</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>PJ Hall</t>
+          <t>Pascal Siakam</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Clemson</t>
+          <t>New Mexico State</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Conference USA</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>Paolo Banchero</t>
+          <t>Pat Connaughton</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Notre Dame</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -6653,148 +6653,148 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>Pascal Siakam</t>
+          <t>Pat Spencer</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>New Mexico State</t>
+          <t>Northwestern</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>C-USA</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>Pat Connaughton</t>
+          <t>Patrick Baldwin Jr.</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Notre Dame</t>
+          <t>Wisconsin-Milwaukee</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Horizon League</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>Pat Spencer</t>
+          <t>Patrick Williams</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Northwestern</t>
+          <t>Florida State</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>Patrick Baldwin Jr.</t>
+          <t>Paul George</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Wisconsin-Milwaukee</t>
+          <t>Fresno State</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>Horizon League</t>
+          <t>Mountain West</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>Patrick Williams</t>
+          <t>Paul Reed</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Florida State</t>
+          <t>DePaul</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>Paul George</t>
+          <t>Payton Pritchard</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Fresno State</t>
+          <t>Oregon</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Mountain West</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>Paul Reed</t>
+          <t>Payton Sandfort</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>DePaul</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>Payton Pritchard</t>
+          <t>Pelle Larsson</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Oregon</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>Payton Sandfort</t>
+          <t>Pete Nance</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>Northwestern</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -6806,177 +6806,177 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>Pelle Larsson</t>
+          <t>Peyton Watson</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>Pete Nance</t>
+          <t>Precious Achiuwa</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Northwestern</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>Peyton Watson</t>
+          <t>Quentin Grimes</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>Precious Achiuwa</t>
+          <t>Quenton Jackson</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Texas A&amp;M</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>AAC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>Quentin Grimes</t>
+          <t>Quinten Post</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Boston College</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>Quenton Jackson</t>
+          <t>RJ Barrett</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>Texas A&amp;M</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>Quinten Post</t>
+          <t>Rasheer Fleming</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>Boston College</t>
+          <t>St. Joseph's (PA)</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Atlantic 10</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>RJ Barrett</t>
+          <t>RayJ Dennis</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Baylor</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>Rasheer Fleming</t>
+          <t>Reed Sheppard</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>St. Joseph's (PA)</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Atlantic 10</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>RayJ Dennis</t>
+          <t>Riley Minix</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Baylor</t>
+          <t>Morehead State</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Ohio Valley</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>Reed Sheppard</t>
+          <t>Rob Dillingham</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
@@ -6993,318 +6993,318 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>Riley Minix</t>
+          <t>Robert Williams III</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Morehead State</t>
+          <t>Texas A&amp;M</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Ohio Valley</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>Rob Dillingham</t>
+          <t>Ron Harper Jr.</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Rutgers</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>Robert Williams III</t>
+          <t>Royce O'Neale</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Texas A&amp;M</t>
+          <t>Baylor</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>Ron Harper Jr.</t>
+          <t>Rui Hachimura</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Rutgers</t>
+          <t>Gonzaga</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>Royce O'Neale</t>
+          <t>Russell Westbrook</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Baylor</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>Rui Hachimura</t>
+          <t>Ryan Dunn</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Gonzaga</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>Russell Westbrook</t>
+          <t>Ryan Kalkbrenner</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Creighton</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>Ryan Dunn</t>
+          <t>Ryan Nembhard</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Gonzaga</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>Ryan Kalkbrenner</t>
+          <t>Ryan Rollins</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Creighton</t>
+          <t>Toledo</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Mid-American</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>Ryan Nembhard</t>
+          <t>Saddiq Bey</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Gonzaga</t>
+          <t>Villanova</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>Ryan Rollins</t>
+          <t>Sam Hauser</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Toledo</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Mid-American</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>Saddiq Bey</t>
+          <t>Sam Merrill</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Villanova</t>
+          <t>Utah State</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Pac-12</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>Sam Hauser</t>
+          <t>Sandro Mamukelashvili</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Seton Hall</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>Sam Merrill</t>
+          <t>Santi Aldama</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Utah State</t>
+          <t>Loyola-Maryland</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Pac-12</t>
+          <t>Patriot League</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>Sandro Mamukelashvili</t>
+          <t>Scottie Barnes</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Seton Hall</t>
+          <t>Florida State</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>Santi Aldama</t>
+          <t>Scotty Pippen Jr.</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Loyola-Maryland</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Patriot League</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>Scottie Barnes</t>
+          <t>Sean Pedulla</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Florida State</t>
+          <t>Mississippi</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>Scotty Pippen Jr.</t>
+          <t>Seth Curry</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>Sean Pedulla</t>
+          <t>Shaedon Sharpe</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>Mississippi</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -7316,29 +7316,29 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>Seth Curry</t>
+          <t>Shai Gilgeous-Alexander</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>Shaedon Sharpe</t>
+          <t>Sharife Cooper</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Auburn</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -7350,250 +7350,250 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>Shai Gilgeous-Alexander</t>
+          <t>Sion James</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>Sharife Cooper</t>
+          <t>Spencer Jones</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Auburn</t>
+          <t>Stanford</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>Sion James</t>
+          <t>Stephen Curry</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Davidson</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Atlantic 10</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>Spencer Jones</t>
+          <t>Stephon Castle</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Stanford</t>
+          <t>Connecticut</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>Stephen Curry</t>
+          <t>Steven Adams</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>Davidson</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Atlantic 10</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>Stephon Castle</t>
+          <t>Svi Mykhailiuk</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>Connecticut</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>Steven Adams</t>
+          <t>T.J. McConnell</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>Svi Mykhailiuk</t>
+          <t>Taelon Peter</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Liberty</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Conference USA</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>T.J. McConnell</t>
+          <t>Taj Gibson</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>USC</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>Taelon Peter</t>
+          <t>Tari Eason</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Liberty</t>
+          <t>LSU</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Conference USA</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>Taj Gibson</t>
+          <t>Taurean Prince</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>USC</t>
+          <t>Baylor</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>Tari Eason</t>
+          <t>Taylor Hendricks</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>LSU</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>Taurean Prince</t>
+          <t>Terance Mann</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Baylor</t>
+          <t>Florida State</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>Taylor Hendricks</t>
+          <t>Terrence Shannon Jr.</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>Illinois</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>Terance Mann</t>
+          <t>Terry Rozier</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Florida State</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -7605,12 +7605,12 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>Terrence Shannon Jr.</t>
+          <t>Thomas Bryant</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Illinois</t>
+          <t>Indiana</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -7622,29 +7622,29 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>Terry Rozier</t>
+          <t>Thomas Sorber</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Georgetown</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>Thomas Bryant</t>
+          <t>Tim Hardaway Jr.</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Michigan</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -7656,114 +7656,114 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>Thomas Sorber</t>
+          <t>Tobias Harris</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Georgetown</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>Tim Hardaway Jr.</t>
+          <t>Tolu Smith</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Mississippi State</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>Tobias Harris</t>
+          <t>Tosan Evbuomwan</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>Princeton</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Ivy League</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>Tolu Smith</t>
+          <t>Toumani Camara</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Mississippi State</t>
+          <t>Dayton</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Atlantic 10</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>Tosan Evbuomwan</t>
+          <t>Trae Young</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>Princeton</t>
+          <t>Oklahoma</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>Ivy League</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>Toumani Camara</t>
+          <t>Trayce Jackson-Davis</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>Dayton</t>
+          <t>Indiana</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Atlantic 10</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>Trae Young</t>
+          <t>Tre Johnson</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>Oklahoma</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
@@ -7775,29 +7775,29 @@
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>Trayce Jackson-Davis</t>
+          <t>Tre Jones</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>Tre Johnson</t>
+          <t>Tre Mann</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
@@ -7809,194 +7809,194 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>Tre Jones</t>
+          <t>Trendon Watford</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>LSU</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>Tre Mann</t>
+          <t>Trevor Keels</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>Trendon Watford</t>
+          <t>Trey Alexander</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>LSU</t>
+          <t>Creighton</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>Trevor Keels</t>
+          <t>Trey Jemison III</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Alabama-Birmingham</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>Trey Alexander</t>
+          <t>Trey Murphy III</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>Creighton</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>Trey Jemison III</t>
+          <t>Tristan Enaruna</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>Alabama-Birmingham</t>
+          <t>Cleveland State</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>American Athletic Conference</t>
+          <t>Horizon League</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>Trey Murphy III</t>
+          <t>Tristan da Silva</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Colorado</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>Tristan Enaruna</t>
+          <t>Tristen Newton</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>Cleveland State</t>
+          <t>Connecticut</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Horizon League</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>Tristan da Silva</t>
+          <t>Ty Jerome</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>Colorado</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>Tristen Newton</t>
+          <t>TyTy Washington Jr.</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>Connecticut</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>Ty Jerome</t>
+          <t>Tyler Burton</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Atlantic 10</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>TyTy Washington Jr.</t>
+          <t>Tyler Herro</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
@@ -8013,46 +8013,46 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>Tyler Burton</t>
+          <t>Tyler Kolek</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Marquette</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>Atlantic 10</t>
+          <t>Big East</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>Tyler Herro</t>
+          <t>Tyrese Haliburton</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Iowa State</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>Tyler Kolek</t>
+          <t>Tyrese Martin</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>Marquette</t>
+          <t>Connecticut</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -8064,58 +8064,58 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>Tyrese Haliburton</t>
+          <t>Tyrese Maxey</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>Iowa State</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>Tyrese Martin</t>
+          <t>Tyrese Proctor</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>Connecticut</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>Big East</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>Tyrese Maxey</t>
+          <t>Tyson Etienne</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Wichita State</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>American Athletic Conference</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>Tyrese Proctor</t>
+          <t>Tyus Jones</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
@@ -8132,165 +8132,165 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>Tyson Etienne</t>
+          <t>VJ Edgecombe</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>Wichita State</t>
+          <t>Baylor</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>AAC</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>Tyus Jones</t>
+          <t>Vladislav Goldin</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Michigan</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>VJ Edgecombe</t>
+          <t>Walker Kessler</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>Baylor</t>
+          <t>Auburn</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>Vladislav Goldin</t>
+          <t>Walter Clayton Jr.</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>Walker Kessler</t>
+          <t>Wendell Carter Jr.</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>Auburn</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>Walter Clayton Jr.</t>
+          <t>Wendell Moore Jr.</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>Wendell Carter Jr.</t>
+          <t>Will Richard</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SEC</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>Wendell Moore Jr.</t>
+          <t>Will Riley</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Illinois</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>Will Richard</t>
+          <t>Xavier Tillman</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Michigan State</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>Will Riley</t>
+          <t>Yanic Konan Niederhäuser</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>Illinois</t>
+          <t>Penn State</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
@@ -8302,168 +8302,134 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>Xavier Tillman</t>
+          <t>Yves Missi</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>Michigan State</t>
+          <t>Baylor</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>Yanic Konan Niederhäuser</t>
+          <t>Zach Collins</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>Penn State</t>
+          <t>Gonzaga</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>West Coast Conference</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>Yves Missi</t>
+          <t>Zach Edey</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>Baylor</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>Zach Collins</t>
+          <t>Zach LaVine</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>Gonzaga</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>Big Ten</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>Zach Edey</t>
+          <t>Zeke Nnaji</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>Big 12</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>Zach LaVine</t>
+          <t>Ziaire Williams</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Stanford</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>Big Ten</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>Zeke Nnaji</t>
+          <t>Zion Williamson</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>Big 12</t>
+          <t>ACC</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>Ziaire Williams</t>
+          <t>Zyon Pullin</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>Stanford</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
-        <is>
-          <t>ACC</t>
-        </is>
-      </c>
-    </row>
-    <row r="472">
-      <c r="A472" t="inlineStr">
-        <is>
-          <t>Zion Williamson</t>
-        </is>
-      </c>
-      <c r="B472" t="inlineStr">
-        <is>
-          <t>Duke</t>
-        </is>
-      </c>
-      <c r="C472" t="inlineStr">
-        <is>
-          <t>ACC</t>
-        </is>
-      </c>
-    </row>
-    <row r="473">
-      <c r="A473" t="inlineStr">
-        <is>
-          <t>Zyon Pullin</t>
-        </is>
-      </c>
-      <c r="B473" t="inlineStr">
-        <is>
-          <t>Florida</t>
-        </is>
-      </c>
-      <c r="C473" t="inlineStr">
         <is>
           <t>SEC</t>
         </is>

</xml_diff>